<commit_message>
rectification erreur et ajout des autres exports
</commit_message>
<xml_diff>
--- a/FILES/VENTE_PAR_CATEGORIE/category-sales-summary-2026-10-01-2026-10-01.xlsx
+++ b/FILES/VENTE_PAR_CATEGORIE/category-sales-summary-2026-10-01-2026-10-01.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FANOMEZANA\PROJETS\APPLICATION_SERVICE_STATION\FILES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FANOMEZANA\PROJETS\NOUVEAUX_RECAP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F3FC088-8D22-41E1-85FE-764C4A2A00F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A9674352-7103-418A-A1A2-B4D08F4FEFD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="14880" xr2:uid="{3BBF3A61-44A1-4AA2-938B-E049C88AD2D8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="14880" xr2:uid="{E2234D57-9FA0-447D-B819-D2DADE2DDE5A}"/>
   </bookViews>
   <sheets>
     <sheet name="category-sales-summary-2026-10-" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,9 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="27">
   <si>
+    <t>CatÃ©gorie</t>
+  </si>
+  <si>
     <t>Articles vendus</t>
   </si>
   <si>
@@ -98,9 +101,6 @@
   </si>
   <si>
     <t>24.000</t>
-  </si>
-  <si>
-    <t>CatÃ©gorie</t>
   </si>
 </sst>
 </file>
@@ -961,69 +961,57 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84BB4AB3-06B1-48D9-9833-9F8FA369AA76}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{526D912B-7C2E-4659-B2BC-186349A406AE}">
   <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="27.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2">
         <v>298000</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1049,16 +1037,16 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3">
         <v>1688500</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1084,16 +1072,16 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C4">
         <v>1175000</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1119,16 +1107,16 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C5">
         <v>585000</v>
       </c>
       <c r="D5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -1154,16 +1142,16 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C6">
         <v>0</v>
       </c>
       <c r="D6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -1189,16 +1177,16 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C7">
         <v>20000</v>
       </c>
       <c r="D7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -1224,16 +1212,16 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C8">
         <v>130000</v>
       </c>
       <c r="D8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -1259,16 +1247,16 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C9">
         <v>114000</v>
       </c>
       <c r="D9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E9">
         <v>0</v>

</xml_diff>